<commit_message>
Update model results and project data
</commit_message>
<xml_diff>
--- a/Capstone Project Docs/Data Dictionary.xlsx
+++ b/Capstone Project Docs/Data Dictionary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/48b30c63d0d95b74/Desktop/Capstone project/Capston Project Docs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/48b30c63d0d95b74/Desktop/Capstone project/Capstone Project Docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="165" documentId="13_ncr:1_{282B82DF-C7A1-4CA4-B556-1481D23E49BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8B745BD1-5ED8-469B-9215-F0E30AA60671}"/>
+  <xr:revisionPtr revIDLastSave="282" documentId="13_ncr:1_{282B82DF-C7A1-4CA4-B556-1481D23E49BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6E457691-E55D-4139-A884-ECA99CA06E4A}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{B0B44A6E-8CE6-4B77-8796-16E0880B61B8}"/>
+    <workbookView minimized="1" xWindow="5760" yWindow="3720" windowWidth="17280" windowHeight="9960" xr2:uid="{B0B44A6E-8CE6-4B77-8796-16E0880B61B8}"/>
   </bookViews>
   <sheets>
     <sheet name="Census Data " sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2289" uniqueCount="1298">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2294" uniqueCount="1298">
   <si>
     <t xml:space="preserve">Variable </t>
   </si>
@@ -4123,7 +4123,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="18">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -4340,11 +4340,31 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
@@ -4389,12 +4409,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -4419,11 +4433,350 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="19" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="58">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="0" tint="-0.14999847407452621"/>
+          <bgColor theme="0" tint="-0.14999847407452621"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color theme="1"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="0" tint="-0.14999847407452621"/>
+          <bgColor theme="0" tint="-0.14999847407452621"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="0" tint="-0.14999847407452621"/>
+          <bgColor theme="0" tint="-0.14999847407452621"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="0" tint="-0.14999847407452621"/>
+          <bgColor theme="0" tint="-0.14999847407452621"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="0" tint="-0.14999847407452621"/>
+          <bgColor theme="0" tint="-0.14999847407452621"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <bottom style="thin">
+          <color theme="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="0" tint="-0.14999847407452621"/>
+          <bgColor theme="0" tint="-0.14999847407452621"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color theme="1"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <bottom style="thin">
+          <color theme="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -5210,332 +5563,6 @@
         </patternFill>
       </fill>
     </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="0" tint="-0.14999847407452621"/>
-          <bgColor theme="0" tint="-0.14999847407452621"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color theme="1"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="0" tint="-0.14999847407452621"/>
-          <bgColor theme="0" tint="-0.14999847407452621"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="0" tint="-0.14999847407452621"/>
-          <bgColor theme="0" tint="-0.14999847407452621"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="0" tint="-0.14999847407452621"/>
-          <bgColor theme="0" tint="-0.14999847407452621"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="0" tint="-0.14999847407452621"/>
-          <bgColor theme="0" tint="-0.14999847407452621"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <bottom style="thin">
-          <color theme="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="0" tint="-0.14999847407452621"/>
-          <bgColor theme="0" tint="-0.14999847407452621"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color theme="1"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <bottom style="thin">
-          <color theme="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -5555,62 +5582,58 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4262A55A-4A45-4A61-B3A9-03993DEA1905}" name="Table2" displayName="Table2" ref="D2:I9" totalsRowShown="0" headerRowDxfId="48" headerRowBorderDxfId="47" tableBorderDxfId="46">
-  <autoFilter ref="D2:I9" xr:uid="{4262A55A-4A45-4A61-B3A9-03993DEA1905}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4262A55A-4A45-4A61-B3A9-03993DEA1905}" name="Table2" displayName="Table2" ref="D2:I11" totalsRowShown="0" headerRowDxfId="8" headerRowBorderDxfId="6" tableBorderDxfId="7">
+  <autoFilter ref="D2:I11" xr:uid="{4262A55A-4A45-4A61-B3A9-03993DEA1905}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{ED1D293D-868A-48CB-8935-7CD2CC172FAD}" name="Variable Name " dataDxfId="45"/>
-    <tableColumn id="2" xr3:uid="{841C3DBD-9B22-4111-A335-2CF56B287EB3}" name="Variable " dataDxfId="44"/>
-    <tableColumn id="7" xr3:uid="{BE1F0E3F-4897-4353-AE4A-E2CE8637387A}" name="Final Name  " dataDxfId="43"/>
-    <tableColumn id="3" xr3:uid="{A351A61F-136F-4C9D-985D-037C47956C0C}" name="Measurment Unit " dataDxfId="42"/>
-    <tableColumn id="4" xr3:uid="{D2F7BA40-0BFC-4C71-983B-AE68EC50511A}" name="Allowed Values " dataDxfId="41"/>
-    <tableColumn id="5" xr3:uid="{14DCD1EB-0412-4582-B31C-4C1CEA63CA74}" name="Description " dataDxfId="40"/>
+    <tableColumn id="1" xr3:uid="{ED1D293D-868A-48CB-8935-7CD2CC172FAD}" name="Variable Name " dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{841C3DBD-9B22-4111-A335-2CF56B287EB3}" name="Variable " dataDxfId="4"/>
+    <tableColumn id="7" xr3:uid="{BE1F0E3F-4897-4353-AE4A-E2CE8637387A}" name="Final Name  " dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{A351A61F-136F-4C9D-985D-037C47956C0C}" name="Measurment Unit " dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{D2F7BA40-0BFC-4C71-983B-AE68EC50511A}" name="Allowed Values " dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{14DCD1EB-0412-4582-B31C-4C1CEA63CA74}" name="Description " dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{421F60A4-5192-4DFE-896C-B0D6AB7FD436}" name="Table7" displayName="Table7" ref="E20:I387" totalsRowShown="0" headerRowDxfId="39" dataDxfId="38">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{421F60A4-5192-4DFE-896C-B0D6AB7FD436}" name="Table7" displayName="Table7" ref="E20:I387" totalsRowShown="0" headerRowDxfId="57" dataDxfId="56">
   <autoFilter ref="E20:I387" xr:uid="{421F60A4-5192-4DFE-896C-B0D6AB7FD436}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{C2C8155E-D4F7-44F1-8B4C-6AC5E1F2DB70}" name="Variable Name " dataDxfId="37"/>
-    <tableColumn id="2" xr3:uid="{4A2C43C6-9D06-4A92-87D8-3EC6DF8BAE7B}" name="Variable" dataDxfId="36"/>
-    <tableColumn id="3" xr3:uid="{4F2341B3-EADD-4051-A904-C2CF40893DF6}" name="Measument Unit " dataDxfId="35"/>
-    <tableColumn id="4" xr3:uid="{E59C00B2-314E-4060-99BF-84015A4C7D75}" name="Allowed Values " dataDxfId="34"/>
-    <tableColumn id="5" xr3:uid="{278E6945-D5DF-4D57-8814-92173882F0B5}" name="Description " dataDxfId="33"/>
+    <tableColumn id="1" xr3:uid="{C2C8155E-D4F7-44F1-8B4C-6AC5E1F2DB70}" name="Variable Name " dataDxfId="55"/>
+    <tableColumn id="2" xr3:uid="{4A2C43C6-9D06-4A92-87D8-3EC6DF8BAE7B}" name="Variable" dataDxfId="54"/>
+    <tableColumn id="3" xr3:uid="{4F2341B3-EADD-4051-A904-C2CF40893DF6}" name="Measument Unit " dataDxfId="53"/>
+    <tableColumn id="4" xr3:uid="{E59C00B2-314E-4060-99BF-84015A4C7D75}" name="Allowed Values " dataDxfId="52"/>
+    <tableColumn id="5" xr3:uid="{278E6945-D5DF-4D57-8814-92173882F0B5}" name="Description " dataDxfId="51"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{B248124D-448B-4560-8672-B866DC45FAB4}" name="Table3" displayName="Table3" ref="B2:G7" totalsRowShown="0" headerRowDxfId="32" headerRowBorderDxfId="31" tableBorderDxfId="30" totalsRowBorderDxfId="29">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{B248124D-448B-4560-8672-B866DC45FAB4}" name="Table3" displayName="Table3" ref="B2:G7" totalsRowShown="0" headerRowDxfId="50" headerRowBorderDxfId="49" tableBorderDxfId="48" totalsRowBorderDxfId="47">
   <autoFilter ref="B2:G7" xr:uid="{B248124D-448B-4560-8672-B866DC45FAB4}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{8E258F16-ECBB-45C0-8A36-D8EB9C0418B8}" name="Variable " dataDxfId="28"/>
-    <tableColumn id="2" xr3:uid="{EEADAC67-4753-4DFE-AB47-96D2A31F4367}" name="Variable Name " dataDxfId="27"/>
-    <tableColumn id="6" xr3:uid="{2D6720DE-2641-44CB-A72E-73A6DBD755E6}" name="Final Name " dataDxfId="26"/>
-    <tableColumn id="3" xr3:uid="{CF5E6454-5456-4543-9E9C-83726F02ACB1}" name="Measurment Unit " dataDxfId="25"/>
-    <tableColumn id="4" xr3:uid="{8F001086-739B-4BC6-9D1C-74BEB08DF231}" name="Allowed Values " dataDxfId="24"/>
-    <tableColumn id="5" xr3:uid="{BD0C6B74-9ED2-45B7-85A4-5B02877ECDD4}" name="Description " dataDxfId="23"/>
+    <tableColumn id="1" xr3:uid="{8E258F16-ECBB-45C0-8A36-D8EB9C0418B8}" name="Variable " dataDxfId="46"/>
+    <tableColumn id="2" xr3:uid="{EEADAC67-4753-4DFE-AB47-96D2A31F4367}" name="Variable Name " dataDxfId="45"/>
+    <tableColumn id="6" xr3:uid="{2D6720DE-2641-44CB-A72E-73A6DBD755E6}" name="Final Name " dataDxfId="44"/>
+    <tableColumn id="3" xr3:uid="{CF5E6454-5456-4543-9E9C-83726F02ACB1}" name="Measurment Unit " dataDxfId="43"/>
+    <tableColumn id="4" xr3:uid="{8F001086-739B-4BC6-9D1C-74BEB08DF231}" name="Allowed Values " dataDxfId="42"/>
+    <tableColumn id="5" xr3:uid="{BD0C6B74-9ED2-45B7-85A4-5B02877ECDD4}" name="Description " dataDxfId="41"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{D57B11AE-9073-4F72-A9A8-2DC1D45E3437}" name="Table6" displayName="Table6" ref="C11:G35" totalsRowShown="0" dataDxfId="22" tableBorderDxfId="21">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{D57B11AE-9073-4F72-A9A8-2DC1D45E3437}" name="Table6" displayName="Table6" ref="C11:G35" totalsRowShown="0" dataDxfId="40" tableBorderDxfId="39">
   <autoFilter ref="C11:G35" xr:uid="{D57B11AE-9073-4F72-A9A8-2DC1D45E3437}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{8D318C54-BF19-4D57-AFC9-EC1F079EA28A}" name="Variable " dataDxfId="20"/>
-    <tableColumn id="2" xr3:uid="{24742D46-0620-4396-A7B7-25F823E20CB0}" name="Variable Name " dataDxfId="19"/>
-    <tableColumn id="3" xr3:uid="{DE4925B2-8580-46A9-8DFA-1C2889480491}" name="Measurment Unit " dataDxfId="18"/>
-    <tableColumn id="4" xr3:uid="{551F881F-CAE1-43C5-8516-3E6F1F9DD39E}" name="Allowed Values " dataDxfId="17"/>
+    <tableColumn id="1" xr3:uid="{8D318C54-BF19-4D57-AFC9-EC1F079EA28A}" name="Variable " dataDxfId="38"/>
+    <tableColumn id="2" xr3:uid="{24742D46-0620-4396-A7B7-25F823E20CB0}" name="Variable Name " dataDxfId="37"/>
+    <tableColumn id="3" xr3:uid="{DE4925B2-8580-46A9-8DFA-1C2889480491}" name="Measurment Unit " dataDxfId="36"/>
+    <tableColumn id="4" xr3:uid="{551F881F-CAE1-43C5-8516-3E6F1F9DD39E}" name="Allowed Values " dataDxfId="35"/>
     <tableColumn id="5" xr3:uid="{0EFBFBD4-613B-46FF-828F-AEBB261E6AD7}" name="Description"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -5618,43 +5641,43 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{FE29614D-F860-4C35-A466-3DE4B7061EBF}" name="Table4" displayName="Table4" ref="D2:I4" totalsRowShown="0" headerRowDxfId="16" headerRowBorderDxfId="15" tableBorderDxfId="14" totalsRowBorderDxfId="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{FE29614D-F860-4C35-A466-3DE4B7061EBF}" name="Table4" displayName="Table4" ref="D2:I4" totalsRowShown="0" headerRowDxfId="34" headerRowBorderDxfId="33" tableBorderDxfId="32" totalsRowBorderDxfId="31">
   <autoFilter ref="D2:I4" xr:uid="{FE29614D-F860-4C35-A466-3DE4B7061EBF}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{971A60C9-5BAC-4D71-8763-9F1883A6A325}" name="Variable " dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{BB22DA7B-2C31-4B6F-BF0C-87D1AB144A52}" name="Variable Name " dataDxfId="11"/>
-    <tableColumn id="6" xr3:uid="{FFC3FD9D-D92D-4AC8-A0A3-968A5B47F366}" name="Final Name " dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{DF042165-BEDA-49D7-A5CB-1023A283F338}" name="Measurment Unit " dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{0443CD8A-8280-40F4-9761-F093B76CE2B7}" name="Allowed Values " dataDxfId="8"/>
-    <tableColumn id="5" xr3:uid="{644FD5BE-D3AF-41F8-B40C-0215AEA1448C}" name="Description " dataDxfId="7"/>
+    <tableColumn id="1" xr3:uid="{971A60C9-5BAC-4D71-8763-9F1883A6A325}" name="Variable " dataDxfId="30"/>
+    <tableColumn id="2" xr3:uid="{BB22DA7B-2C31-4B6F-BF0C-87D1AB144A52}" name="Variable Name " dataDxfId="29"/>
+    <tableColumn id="6" xr3:uid="{FFC3FD9D-D92D-4AC8-A0A3-968A5B47F366}" name="Final Name " dataDxfId="28"/>
+    <tableColumn id="3" xr3:uid="{DF042165-BEDA-49D7-A5CB-1023A283F338}" name="Measurment Unit " dataDxfId="27"/>
+    <tableColumn id="4" xr3:uid="{0443CD8A-8280-40F4-9761-F093B76CE2B7}" name="Allowed Values " dataDxfId="26"/>
+    <tableColumn id="5" xr3:uid="{644FD5BE-D3AF-41F8-B40C-0215AEA1448C}" name="Description " dataDxfId="25"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D78252BF-0658-4EC7-9851-A0CC2D6A1DBC}" name="Table1" displayName="Table1" ref="E9:I15" totalsRowShown="0" dataDxfId="6" tableBorderDxfId="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D78252BF-0658-4EC7-9851-A0CC2D6A1DBC}" name="Table1" displayName="Table1" ref="E9:I15" totalsRowShown="0" dataDxfId="24" tableBorderDxfId="23">
   <autoFilter ref="E9:I15" xr:uid="{D78252BF-0658-4EC7-9851-A0CC2D6A1DBC}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{546AF41F-96CA-4EB2-B20A-69E45A881228}" name="Variable " dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{C6ADAF7C-14AD-44C2-B679-BA454612E950}" name="Variable Name " dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{49A92D62-0DDB-4EAA-A28A-394EB8F0AB60}" name="Measurmet Unit " dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{E462107F-1E58-4431-96CD-0E4A0955D6C1}" name="Allowed Values " dataDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{9792CDCD-04C2-41E7-87DE-F4585A4730BC}" name="Description " dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{546AF41F-96CA-4EB2-B20A-69E45A881228}" name="Variable " dataDxfId="22"/>
+    <tableColumn id="2" xr3:uid="{C6ADAF7C-14AD-44C2-B679-BA454612E950}" name="Variable Name " dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{49A92D62-0DDB-4EAA-A28A-394EB8F0AB60}" name="Measurmet Unit " dataDxfId="20"/>
+    <tableColumn id="4" xr3:uid="{E462107F-1E58-4431-96CD-0E4A0955D6C1}" name="Allowed Values " dataDxfId="19"/>
+    <tableColumn id="5" xr3:uid="{9792CDCD-04C2-41E7-87DE-F4585A4730BC}" name="Description " dataDxfId="18"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{51BD6F9C-D446-43E5-B23A-D38E849C3DA3}" name="Table5" displayName="Table5" ref="D2:H38" totalsRowShown="0" headerRowDxfId="57" headerRowBorderDxfId="56" tableBorderDxfId="55" totalsRowBorderDxfId="54">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{51BD6F9C-D446-43E5-B23A-D38E849C3DA3}" name="Table5" displayName="Table5" ref="D2:H38" totalsRowShown="0" headerRowDxfId="17" headerRowBorderDxfId="16" tableBorderDxfId="15" totalsRowBorderDxfId="14">
   <autoFilter ref="D2:H38" xr:uid="{51BD6F9C-D446-43E5-B23A-D38E849C3DA3}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{53A8D7B9-8FCF-4F47-8BC3-5345A66A4311}" name="Variable " dataDxfId="53"/>
-    <tableColumn id="2" xr3:uid="{D37222E3-F794-4389-B3F3-019B12E7E76C}" name="Variable Name " dataDxfId="52"/>
-    <tableColumn id="3" xr3:uid="{A51664D5-9678-4BBB-9B62-4D0F25CE9F5A}" name="Measurment Unit " dataDxfId="51"/>
-    <tableColumn id="4" xr3:uid="{99CE2BA3-33CF-4967-8B24-C8449C5C9AF4}" name="Allowed Values " dataDxfId="50"/>
-    <tableColumn id="5" xr3:uid="{96C07542-FAD1-4CA0-AD2D-5D375E2F96A4}" name="Description " dataDxfId="49"/>
+    <tableColumn id="1" xr3:uid="{53A8D7B9-8FCF-4F47-8BC3-5345A66A4311}" name="Variable " dataDxfId="13"/>
+    <tableColumn id="2" xr3:uid="{D37222E3-F794-4389-B3F3-019B12E7E76C}" name="Variable Name " dataDxfId="12"/>
+    <tableColumn id="3" xr3:uid="{A51664D5-9678-4BBB-9B62-4D0F25CE9F5A}" name="Measurment Unit " dataDxfId="11"/>
+    <tableColumn id="4" xr3:uid="{99CE2BA3-33CF-4967-8B24-C8449C5C9AF4}" name="Allowed Values " dataDxfId="10"/>
+    <tableColumn id="5" xr3:uid="{96C07542-FAD1-4CA0-AD2D-5D375E2F96A4}" name="Description " dataDxfId="9"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5989,14 +6012,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="4:9" ht="55.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D1" s="32" t="s">
+      <c r="D1" s="30" t="s">
         <v>1218</v>
       </c>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
-      <c r="G1" s="33"/>
-      <c r="H1" s="33"/>
-      <c r="I1" s="33"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
+      <c r="I1" s="31"/>
     </row>
     <row r="2" spans="4:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D2" s="1" t="s">
@@ -6158,8 +6181,42 @@
         <v>1099</v>
       </c>
     </row>
-    <row r="10" spans="4:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="11" spans="4:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="10" spans="4:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D10" s="41" t="s">
+        <v>792</v>
+      </c>
+      <c r="E10" s="42" t="s">
+        <v>418</v>
+      </c>
+      <c r="F10" s="43"/>
+      <c r="G10" s="43" t="s">
+        <v>34</v>
+      </c>
+      <c r="H10" s="23" t="s">
+        <v>867</v>
+      </c>
+      <c r="I10" s="23" t="s">
+        <v>1151</v>
+      </c>
+    </row>
+    <row r="11" spans="4:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D11" s="41" t="s">
+        <v>534</v>
+      </c>
+      <c r="E11" s="42" t="s">
+        <v>160</v>
+      </c>
+      <c r="F11" s="43"/>
+      <c r="G11" s="43" t="s">
+        <v>34</v>
+      </c>
+      <c r="H11" s="23" t="s">
+        <v>866</v>
+      </c>
+      <c r="I11" s="23" t="s">
+        <v>910</v>
+      </c>
+    </row>
     <row r="12" spans="4:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="13" spans="4:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="4:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -6167,20 +6224,20 @@
     <row r="16" spans="4:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="17" spans="5:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="18" spans="5:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="E18" s="34" t="s">
+      <c r="E18" s="32" t="s">
         <v>1219</v>
       </c>
-      <c r="F18" s="35"/>
-      <c r="G18" s="35"/>
-      <c r="H18" s="35"/>
-      <c r="I18" s="35"/>
+      <c r="F18" s="33"/>
+      <c r="G18" s="33"/>
+      <c r="H18" s="33"/>
+      <c r="I18" s="33"/>
     </row>
     <row r="19" spans="5:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="E19" s="35"/>
-      <c r="F19" s="35"/>
-      <c r="G19" s="35"/>
-      <c r="H19" s="35"/>
-      <c r="I19" s="35"/>
+      <c r="E19" s="33"/>
+      <c r="F19" s="33"/>
+      <c r="G19" s="33"/>
+      <c r="H19" s="33"/>
+      <c r="I19" s="33"/>
     </row>
     <row r="20" spans="5:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="E20" t="s">
@@ -6897,21 +6954,11 @@
       </c>
     </row>
     <row r="62" spans="5:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="E62" s="27" t="s">
-        <v>534</v>
-      </c>
-      <c r="F62" s="28" t="s">
-        <v>160</v>
-      </c>
-      <c r="G62" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="H62" s="1" t="s">
-        <v>866</v>
-      </c>
-      <c r="I62" s="29" t="s">
-        <v>910</v>
-      </c>
+      <c r="E62" s="44"/>
+      <c r="F62" s="45"/>
+      <c r="G62" s="46"/>
+      <c r="H62" s="46"/>
+      <c r="I62" s="40"/>
     </row>
     <row r="63" spans="5:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="E63" s="27" t="s">
@@ -12466,14 +12513,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:7" ht="66.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="36" t="s">
+      <c r="B1" s="34" t="s">
         <v>1213</v>
       </c>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="37"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
     </row>
     <row r="2" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B2" s="6" t="s">
@@ -12596,20 +12643,20 @@
       </c>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="C9" s="38" t="s">
+      <c r="C9" s="36" t="s">
         <v>1212</v>
       </c>
-      <c r="D9" s="39"/>
-      <c r="E9" s="39"/>
-      <c r="F9" s="39"/>
-      <c r="G9" s="39"/>
+      <c r="D9" s="37"/>
+      <c r="E9" s="37"/>
+      <c r="F9" s="37"/>
+      <c r="G9" s="37"/>
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="C10" s="39"/>
-      <c r="D10" s="39"/>
-      <c r="E10" s="39"/>
-      <c r="F10" s="39"/>
-      <c r="G10" s="39"/>
+      <c r="C10" s="37"/>
+      <c r="D10" s="37"/>
+      <c r="E10" s="37"/>
+      <c r="F10" s="37"/>
+      <c r="G10" s="37"/>
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.3">
       <c r="C11" t="s">
@@ -13054,14 +13101,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="4:9" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D1" s="36" t="s">
+      <c r="D1" s="34" t="s">
         <v>92</v>
       </c>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="37"/>
-      <c r="H1" s="37"/>
-      <c r="I1" s="37"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
+      <c r="H1" s="35"/>
+      <c r="I1" s="35"/>
     </row>
     <row r="2" spans="4:9" x14ac:dyDescent="0.3">
       <c r="D2" s="6" t="s">
@@ -13125,21 +13172,21 @@
     </row>
     <row r="7" spans="4:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D7" s="18"/>
-      <c r="E7" s="34" t="s">
+      <c r="E7" s="32" t="s">
         <v>1210</v>
       </c>
-      <c r="F7" s="34"/>
-      <c r="G7" s="34"/>
-      <c r="H7" s="34"/>
-      <c r="I7" s="34"/>
+      <c r="F7" s="32"/>
+      <c r="G7" s="32"/>
+      <c r="H7" s="32"/>
+      <c r="I7" s="32"/>
     </row>
     <row r="8" spans="4:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D8" s="18"/>
-      <c r="E8" s="34"/>
-      <c r="F8" s="34"/>
-      <c r="G8" s="34"/>
-      <c r="H8" s="34"/>
-      <c r="I8" s="34"/>
+      <c r="E8" s="32"/>
+      <c r="F8" s="32"/>
+      <c r="G8" s="32"/>
+      <c r="H8" s="32"/>
+      <c r="I8" s="32"/>
     </row>
     <row r="9" spans="4:9" x14ac:dyDescent="0.3">
       <c r="E9" t="s">
@@ -13286,13 +13333,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="4:8" ht="46.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D1" s="30" t="s">
+      <c r="D1" s="38" t="s">
         <v>1207</v>
       </c>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
-      <c r="H1" s="31"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="39"/>
     </row>
     <row r="2" spans="4:8" x14ac:dyDescent="0.3">
       <c r="D2" s="6" t="s">

</xml_diff>